<commit_message>
Fix reproducible setup and regenerate Q1 to Q6 outputs
</commit_message>
<xml_diff>
--- a/08_tables/between_within_descriptive_statistics.xlsx
+++ b/08_tables/between_within_descriptive_statistics.xlsx
@@ -501,7 +501,7 @@
         <v>48.94083489359494</v>
       </c>
       <c r="F2" t="n">
-        <v>9.633156076217411</v>
+        <v>9.633156076217412</v>
       </c>
       <c r="G2" t="n">
         <v>30.1622622994095</v>
@@ -609,7 +609,7 @@
         <v>-0.4529999999999887</v>
       </c>
       <c r="F5" t="n">
-        <v>4.248727191401601</v>
+        <v>4.248727191401604</v>
       </c>
       <c r="G5" t="n">
         <v>-10.69</v>
@@ -681,7 +681,7 @@
         <v>-0.6655016666666618</v>
       </c>
       <c r="F7" t="n">
-        <v>4.666285623271245</v>
+        <v>4.666285623271247</v>
       </c>
       <c r="G7" t="n">
         <v>-8.394419999999997</v>

</xml_diff>